<commit_message>
Apply Nedra palette (indigo, lime, sky, teal, orange) to HTML, diagrams and Excel
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A9jLsEDeJJYPHEQRo2Ao9x
</commit_message>
<xml_diff>
--- a/docs/release-trz-fte.xlsx
+++ b/docs/release-trz-fte.xlsx
@@ -602,20 +602,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E79"/>
-        <bgColor rgb="FF003366"/>
+        <fgColor rgb="FF140093"/>
+        <bgColor rgb="FF000080"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFE2EFDA"/>
+        <fgColor rgb="FFFFE4CC"/>
+        <bgColor rgb="FFEAFAB8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
-        <bgColor rgb="FFFFF2CC"/>
+        <fgColor rgb="FFEAFAB8"/>
+        <bgColor rgb="FFFFFF99"/>
       </patternFill>
     </fill>
   </fills>
@@ -770,7 +770,7 @@
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF140093"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
@@ -778,7 +778,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF2CC"/>
+      <rgbColor rgb="FFEAFAB8"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -794,12 +794,12 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFE2EFDA"/>
+      <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFFE4CC"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -814,7 +814,7 @@
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF1F4E79"/>
+      <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>

</xml_diff>

<commit_message>
Apply role model cards (FRM): role mapping, decision rights at gates, draft cards, KPI metrics M11-M14, new roles; findings F24-F26
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A9jLsEDeJJYPHEQRo2Ao9x
</commit_message>
<xml_diff>
--- a/docs/release-trz-fte.xlsx
+++ b/docs/release-trz-fte.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="169">
   <si>
     <t xml:space="preserve">Параметр</t>
   </si>
@@ -399,7 +399,13 @@
     <t xml:space="preserve">11.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Уведомление пользователей</t>
+    <t xml:space="preserve">Уведомление пользователей, release notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ТПИ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Технический писатель</t>
   </si>
   <si>
     <t xml:space="preserve">PMM</t>
@@ -448,6 +454,18 @@
   </si>
   <si>
     <t xml:space="preserve">Закрытие релиза и ретро</t>
+  </si>
+  <si>
+    <t xml:space="preserve">СМ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Скрам-мастер</t>
+  </si>
+  <si>
+    <t xml:space="preserve">АП</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Администратор проекта</t>
   </si>
   <si>
     <t xml:space="preserve">Итого</t>
@@ -1164,7 +1182,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K64"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -3020,7 +3038,7 @@
         <v>122</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F48" s="3" t="n">
         <v>0</v>
@@ -3034,15 +3052,15 @@
       </c>
       <c r="I48" s="7" t="n">
         <f aca="false">(E48+F48*N_SVC)*H48</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J48" s="7" t="n">
         <f aca="false">(E48*HF_F+F48)*H48</f>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="K48" s="7" t="n">
         <f aca="false">I48*REL_YEAR+J48*HF_YEAR</f>
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3053,10 +3071,10 @@
         <v>120</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>38</v>
+        <v>123</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>39</v>
+        <v>124</v>
       </c>
       <c r="E49" s="3" t="n">
         <v>1</v>
@@ -3086,22 +3104,22 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>125</v>
+        <v>38</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>126</v>
+        <v>39</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="G50" s="3" t="s">
         <v>40</v>
@@ -3112,35 +3130,35 @@
       </c>
       <c r="I50" s="7" t="n">
         <f aca="false">(E50+F50*N_SVC)*H50</f>
-        <v>6.5</v>
+        <v>1</v>
       </c>
       <c r="J50" s="7" t="n">
         <f aca="false">(E50*HF_F+F50)*H50</f>
-        <v>2.25</v>
+        <v>0.5</v>
       </c>
       <c r="K50" s="7" t="n">
         <f aca="false">I50*REL_YEAR+J50*HF_YEAR</f>
-        <v>87</v>
+        <v>14</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>38</v>
+        <v>127</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>39</v>
+        <v>128</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>40</v>
@@ -3151,35 +3169,35 @@
       </c>
       <c r="I51" s="7" t="n">
         <f aca="false">(E51+F51*N_SVC)*H51</f>
-        <v>3</v>
+        <v>6.5</v>
       </c>
       <c r="J51" s="7" t="n">
         <f aca="false">(E51*HF_F+F51)*H51</f>
-        <v>1.5</v>
+        <v>2.25</v>
       </c>
       <c r="K51" s="7" t="n">
         <f aca="false">I51*REL_YEAR+J51*HF_YEAR</f>
-        <v>42</v>
+        <v>87</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>105</v>
+        <v>38</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>106</v>
+        <v>39</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="G52" s="3" t="s">
         <v>40</v>
@@ -3190,15 +3208,15 @@
       </c>
       <c r="I52" s="7" t="n">
         <f aca="false">(E52+F52*N_SVC)*H52</f>
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="J52" s="7" t="n">
         <f aca="false">(E52*HF_F+F52)*H52</f>
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="K52" s="7" t="n">
         <f aca="false">I52*REL_YEAR+J52*HF_YEAR</f>
-        <v>59</v>
+        <v>42</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3209,10 +3227,10 @@
         <v>130</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E53" s="3" t="n">
         <v>2</v>
@@ -3248,16 +3266,16 @@
         <v>132</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="G54" s="3" t="s">
         <v>40</v>
@@ -3268,15 +3286,15 @@
       </c>
       <c r="I54" s="7" t="n">
         <f aca="false">(E54+F54*N_SVC)*H54</f>
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="J54" s="7" t="n">
         <f aca="false">(E54*HF_F+F54)*H54</f>
-        <v>2.5</v>
+        <v>1.25</v>
       </c>
       <c r="K54" s="7" t="n">
         <f aca="false">I54*REL_YEAR+J54*HF_YEAR</f>
-        <v>118</v>
+        <v>59</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3287,16 +3305,16 @@
         <v>134</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>43</v>
+        <v>113</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>44</v>
+        <v>114</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="G55" s="3" t="s">
         <v>40</v>
@@ -3307,35 +3325,35 @@
       </c>
       <c r="I55" s="7" t="n">
         <f aca="false">(E55+F55*N_SVC)*H55</f>
-        <v>4.5</v>
+        <v>9</v>
       </c>
       <c r="J55" s="7" t="n">
         <f aca="false">(E55*HF_F+F55)*H55</f>
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="K55" s="7" t="n">
         <f aca="false">I55*REL_YEAR+J55*HF_YEAR</f>
-        <v>59</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="G56" s="3" t="s">
         <v>40</v>
@@ -3346,18 +3364,18 @@
       </c>
       <c r="I56" s="7" t="n">
         <f aca="false">(E56+F56*N_SVC)*H56</f>
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="J56" s="7" t="n">
         <f aca="false">(E56*HF_F+F56)*H56</f>
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="K56" s="7" t="n">
         <f aca="false">I56*REL_YEAR+J56*HF_YEAR</f>
-        <v>62</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
         <v>135</v>
       </c>
@@ -3365,16 +3383,16 @@
         <v>136</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>40</v>
@@ -3385,32 +3403,32 @@
       </c>
       <c r="I57" s="7" t="n">
         <f aca="false">(E57+F57*N_SVC)*H57</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J57" s="7" t="n">
         <f aca="false">(E57*HF_F+F57)*H57</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="K57" s="7" t="n">
         <f aca="false">I57*REL_YEAR+J57*HF_YEAR</f>
-        <v>28</v>
+        <v>62</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F58" s="3" t="n">
         <v>0</v>
@@ -3424,32 +3442,32 @@
       </c>
       <c r="I58" s="7" t="n">
         <f aca="false">(E58+F58*N_SVC)*H58</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J58" s="7" t="n">
         <f aca="false">(E58*HF_F+F58)*H58</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K58" s="7" t="n">
         <f aca="false">I58*REL_YEAR+J58*HF_YEAR</f>
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>68</v>
+        <v>139</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>69</v>
+        <v>140</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F59" s="3" t="n">
         <v>0</v>
@@ -3463,35 +3481,35 @@
       </c>
       <c r="I59" s="7" t="n">
         <f aca="false">(E59+F59*N_SVC)*H59</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J59" s="7" t="n">
         <f aca="false">(E59*HF_F+F59)*H59</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K59" s="7" t="n">
         <f aca="false">I59*REL_YEAR+J59*HF_YEAR</f>
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>59</v>
+        <v>141</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>60</v>
+        <v>142</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G60" s="3" t="s">
         <v>40</v>
@@ -3502,39 +3520,156 @@
       </c>
       <c r="I60" s="7" t="n">
         <f aca="false">(E60+F60*N_SVC)*H60</f>
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="J60" s="7" t="n">
         <f aca="false">(E60*HF_F+F60)*H60</f>
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="K60" s="7" t="n">
         <f aca="false">I60*REL_YEAR+J60*HF_YEAR</f>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H61" s="6" t="n">
+        <f aca="false">IF(G61="psi",P_PSI,IF(G61="ptz",P_PTZ,1))</f>
+        <v>1</v>
+      </c>
+      <c r="I61" s="7" t="n">
+        <f aca="false">(E61+F61*N_SVC)*H61</f>
+        <v>1</v>
+      </c>
+      <c r="J61" s="7" t="n">
+        <f aca="false">(E61*HF_F+F61)*H61</f>
+        <v>0.5</v>
+      </c>
+      <c r="K61" s="7" t="n">
+        <f aca="false">I61*REL_YEAR+J61*HF_YEAR</f>
         <v>14</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="2"/>
-      <c r="B61" s="8" t="s">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-      <c r="E61" s="2"/>
-      <c r="F61" s="2"/>
-      <c r="G61" s="2"/>
-      <c r="H61" s="6"/>
-      <c r="I61" s="9" t="n">
-        <f aca="false">SUM(I2:I60)</f>
-        <v>635.5</v>
-      </c>
-      <c r="J61" s="9" t="n">
-        <f aca="false">SUM(J2:J60)</f>
-        <v>124.35</v>
-      </c>
-      <c r="K61" s="9" t="n">
-        <f aca="false">SUM(K2:K60)</f>
-        <v>8123.4</v>
+      <c r="B62" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H62" s="6" t="n">
+        <f aca="false">IF(G62="psi",P_PSI,IF(G62="ptz",P_PTZ,1))</f>
+        <v>1</v>
+      </c>
+      <c r="I62" s="7" t="n">
+        <f aca="false">(E62+F62*N_SVC)*H62</f>
+        <v>1</v>
+      </c>
+      <c r="J62" s="7" t="n">
+        <f aca="false">(E62*HF_F+F62)*H62</f>
+        <v>0.5</v>
+      </c>
+      <c r="K62" s="7" t="n">
+        <f aca="false">I62*REL_YEAR+J62*HF_YEAR</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H63" s="6" t="n">
+        <f aca="false">IF(G63="psi",P_PSI,IF(G63="ptz",P_PTZ,1))</f>
+        <v>1</v>
+      </c>
+      <c r="I63" s="7" t="n">
+        <f aca="false">(E63+F63*N_SVC)*H63</f>
+        <v>1</v>
+      </c>
+      <c r="J63" s="7" t="n">
+        <f aca="false">(E63*HF_F+F63)*H63</f>
+        <v>0.5</v>
+      </c>
+      <c r="K63" s="7" t="n">
+        <f aca="false">I63*REL_YEAR+J63*HF_YEAR</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="2"/>
+      <c r="B64" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="C64" s="2"/>
+      <c r="D64" s="2"/>
+      <c r="E64" s="2"/>
+      <c r="F64" s="2"/>
+      <c r="G64" s="2"/>
+      <c r="H64" s="6"/>
+      <c r="I64" s="9" t="n">
+        <f aca="false">SUM(I2:I63)</f>
+        <v>644</v>
+      </c>
+      <c r="J64" s="9" t="n">
+        <f aca="false">SUM(J2:J63)</f>
+        <v>127.6</v>
+      </c>
+      <c r="K64" s="9" t="n">
+        <f aca="false">SUM(K2:K63)</f>
+        <v>8238.4</v>
       </c>
     </row>
   </sheetData>
@@ -3553,7 +3688,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -3582,25 +3717,25 @@
         <v>35</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3611,11 +3746,11 @@
         <v>39</v>
       </c>
       <c r="C2" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$60,'ТРЗ по шагам'!$C$2:$C$60,A2)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A2)</f>
         <v>51.5</v>
       </c>
       <c r="D2" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$60,'ТРЗ по шагам'!$C$2:$C$60,A2)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A2)</f>
         <v>699.4</v>
       </c>
       <c r="E2" s="6" t="n">
@@ -3651,11 +3786,11 @@
         <v>44</v>
       </c>
       <c r="C3" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$60,'ТРЗ по шагам'!$C$2:$C$60,A3)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A3)</f>
         <v>58.5</v>
       </c>
       <c r="D3" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$60,'ТРЗ по шагам'!$C$2:$C$60,A3)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A3)</f>
         <v>771</v>
       </c>
       <c r="E3" s="6" t="n">
@@ -3691,11 +3826,11 @@
         <v>46</v>
       </c>
       <c r="C4" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$60,'ТРЗ по шагам'!$C$2:$C$60,A4)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A4)</f>
         <v>234</v>
       </c>
       <c r="D4" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$60,'ТРЗ по шагам'!$C$2:$C$60,A4)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A4)</f>
         <v>2908</v>
       </c>
       <c r="E4" s="6" t="n">
@@ -3731,11 +3866,11 @@
         <v>98</v>
       </c>
       <c r="C5" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$60,'ТРЗ по шагам'!$C$2:$C$60,A5)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A5)</f>
         <v>13</v>
       </c>
       <c r="D5" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$60,'ТРЗ по шагам'!$C$2:$C$60,A5)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A5)</f>
         <v>174</v>
       </c>
       <c r="E5" s="6" t="n">
@@ -3771,11 +3906,11 @@
         <v>69</v>
       </c>
       <c r="C6" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$60,'ТРЗ по шагам'!$C$2:$C$60,A6)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A6)</f>
         <v>167</v>
       </c>
       <c r="D6" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$60,'ТРЗ по шагам'!$C$2:$C$60,A6)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A6)</f>
         <v>2106</v>
       </c>
       <c r="E6" s="6" t="n">
@@ -3811,11 +3946,11 @@
         <v>71</v>
       </c>
       <c r="C7" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$60,'ТРЗ по шагам'!$C$2:$C$60,A7)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A7)</f>
         <v>3</v>
       </c>
       <c r="D7" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$60,'ТРЗ по шагам'!$C$2:$C$60,A7)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A7)</f>
         <v>42</v>
       </c>
       <c r="E7" s="6" t="n">
@@ -3851,11 +3986,11 @@
         <v>87</v>
       </c>
       <c r="C8" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$60,'ТРЗ по шагам'!$C$2:$C$60,A8)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A8)</f>
         <v>2</v>
       </c>
       <c r="D8" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$60,'ТРЗ по шагам'!$C$2:$C$60,A8)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A8)</f>
         <v>28</v>
       </c>
       <c r="E8" s="6" t="n">
@@ -3885,29 +4020,29 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C9" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$60,'ТРЗ по шагам'!$C$2:$C$60,A9)</f>
-        <v>3</v>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A9)</f>
+        <v>1</v>
       </c>
       <c r="D9" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$60,'ТРЗ по шагам'!$C$2:$C$60,A9)</f>
-        <v>42</v>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A9)</f>
+        <v>14</v>
       </c>
       <c r="E9" s="6" t="n">
         <f aca="false">D9/H_FTE</f>
-        <v>0.0265688259109312</v>
+        <v>0.00885627530364372</v>
       </c>
       <c r="F9" s="11" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="6" t="n">
         <f aca="false">F9-E9</f>
-        <v>0.973431174089069</v>
+        <v>0.991143724696356</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="12" t="str">
@@ -3931,11 +4066,11 @@
         <v>60</v>
       </c>
       <c r="C10" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$60,'ТРЗ по шагам'!$C$2:$C$60,A10)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A10)</f>
         <v>37</v>
       </c>
       <c r="D10" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$60,'ТРЗ по шагам'!$C$2:$C$60,A10)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A10)</f>
         <v>490</v>
       </c>
       <c r="E10" s="6" t="n">
@@ -3965,17 +4100,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C11" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$60,'ТРЗ по шагам'!$C$2:$C$60,A11)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A11)</f>
         <v>6.5</v>
       </c>
       <c r="D11" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$60,'ТРЗ по шагам'!$C$2:$C$60,A11)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A11)</f>
         <v>87</v>
       </c>
       <c r="E11" s="6" t="n">
@@ -4011,11 +4146,11 @@
         <v>114</v>
       </c>
       <c r="C12" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$60,'ТРЗ по шагам'!$C$2:$C$60,A12)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A12)</f>
         <v>37</v>
       </c>
       <c r="D12" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$60,'ТРЗ по шагам'!$C$2:$C$60,A12)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A12)</f>
         <v>478</v>
       </c>
       <c r="E12" s="6" t="n">
@@ -4051,11 +4186,11 @@
         <v>106</v>
       </c>
       <c r="C13" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$60,'ТРЗ по шагам'!$C$2:$C$60,A13)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A13)</f>
         <v>11.5</v>
       </c>
       <c r="D13" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$60,'ТРЗ по шагам'!$C$2:$C$60,A13)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A13)</f>
         <v>149</v>
       </c>
       <c r="E13" s="6" t="n">
@@ -4091,11 +4226,11 @@
         <v>110</v>
       </c>
       <c r="C14" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$60,'ТРЗ по шагам'!$C$2:$C$60,A14)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A14)</f>
         <v>11.5</v>
       </c>
       <c r="D14" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$60,'ТРЗ по шагам'!$C$2:$C$60,A14)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A14)</f>
         <v>149</v>
       </c>
       <c r="E14" s="6" t="n">
@@ -4124,47 +4259,167 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2"/>
-      <c r="B15" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="C15" s="13" t="n">
-        <f aca="false">SUM(C2:C14)</f>
-        <v>635.5</v>
-      </c>
-      <c r="D15" s="13" t="n">
-        <f aca="false">SUM(D2:D14)</f>
-        <v>8123.4</v>
-      </c>
-      <c r="E15" s="14" t="n">
-        <f aca="false">SUM(E2:E14)</f>
-        <v>5.13879048582996</v>
-      </c>
-      <c r="F15" s="14" t="n">
-        <f aca="false">SUM(F2:F14)</f>
-        <v>13</v>
-      </c>
-      <c r="G15" s="14" t="n">
-        <f aca="false">SUM(G2:G14)</f>
-        <v>7.86120951417004</v>
-      </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="15" t="n">
-        <f aca="false">SUM(I2:I14)</f>
+      <c r="A15" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A15)</f>
+        <v>2</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A15)</f>
+        <v>28</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <f aca="false">D15/H_FTE</f>
+        <v>0.0177125506072874</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <f aca="false">F15-E15</f>
+        <v>0.982287449392713</v>
+      </c>
+      <c r="H15" s="3"/>
+      <c r="I15" s="12" t="str">
+        <f aca="false">IF(H15="","",D15*H15)</f>
+        <v/>
+      </c>
+      <c r="J15" s="12" t="str">
+        <f aca="false">IF(H15="","",F15*H_FULL*H15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="12" t="str">
+        <f aca="false">IF(H15="","",J15-I15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A16)</f>
+        <v>4.5</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A16)</f>
+        <v>59</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <f aca="false">D16/H_FTE</f>
+        <v>0.0373228744939271</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <f aca="false">F16-E16</f>
+        <v>0.962677125506073</v>
+      </c>
+      <c r="H16" s="3"/>
+      <c r="I16" s="12" t="str">
+        <f aca="false">IF(H16="","",D16*H16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="12" t="str">
+        <f aca="false">IF(H16="","",F16*H_FULL*H16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="12" t="str">
+        <f aca="false">IF(H16="","",J16-I16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A17)</f>
+        <v>4</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A17)</f>
+        <v>56</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <f aca="false">D17/H_FTE</f>
+        <v>0.0354251012145749</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <f aca="false">F17-E17</f>
+        <v>0.964574898785425</v>
+      </c>
+      <c r="H17" s="3"/>
+      <c r="I17" s="12" t="str">
+        <f aca="false">IF(H17="","",D17*H17)</f>
+        <v/>
+      </c>
+      <c r="J17" s="12" t="str">
+        <f aca="false">IF(H17="","",F17*H_FULL*H17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="12" t="str">
+        <f aca="false">IF(H17="","",J17-I17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2"/>
+      <c r="B18" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="C18" s="13" t="n">
+        <f aca="false">SUM(C2:C17)</f>
+        <v>644</v>
+      </c>
+      <c r="D18" s="13" t="n">
+        <f aca="false">SUM(D2:D17)</f>
+        <v>8238.4</v>
+      </c>
+      <c r="E18" s="14" t="n">
+        <f aca="false">SUM(E2:E17)</f>
+        <v>5.21153846153846</v>
+      </c>
+      <c r="F18" s="14" t="n">
+        <f aca="false">SUM(F2:F17)</f>
+        <v>16</v>
+      </c>
+      <c r="G18" s="14" t="n">
+        <f aca="false">SUM(G2:G17)</f>
+        <v>10.7884615384615</v>
+      </c>
+      <c r="H18" s="2"/>
+      <c r="I18" s="15" t="n">
+        <f aca="false">SUM(I2:I17)</f>
         <v>0</v>
       </c>
-      <c r="J15" s="15" t="n">
-        <f aca="false">SUM(J2:J14)</f>
+      <c r="J18" s="15" t="n">
+        <f aca="false">SUM(J2:J17)</f>
         <v>0</v>
       </c>
-      <c r="K15" s="15" t="n">
-        <f aca="false">SUM(K2:K14)</f>
+      <c r="K18" s="15" t="n">
+        <f aca="false">SUM(K2:K17)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
-        <v>145</v>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -4183,7 +4438,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -4199,24 +4454,24 @@
         <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C2" s="16" t="n">
         <v>5</v>
@@ -4242,23 +4497,23 @@
         <v>39</v>
       </c>
       <c r="C3" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.391194331983806</v>
       </c>
       <c r="D3" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.442434210526316</v>
       </c>
       <c r="E3" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.493674089068826</v>
       </c>
       <c r="F3" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.544913967611336</v>
       </c>
       <c r="G3" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A3)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.596153846153846</v>
       </c>
     </row>
@@ -4270,23 +4525,23 @@
         <v>44</v>
       </c>
       <c r="C4" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.373861336032389</v>
       </c>
       <c r="D4" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.487727732793522</v>
       </c>
       <c r="E4" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.601594129554656</v>
       </c>
       <c r="F4" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.715460526315789</v>
       </c>
       <c r="G4" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A4)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.829326923076923</v>
       </c>
     </row>
@@ -4298,23 +4553,23 @@
         <v>46</v>
       </c>
       <c r="C5" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.966599190283401</v>
       </c>
       <c r="D5" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>1.83957489878542</v>
       </c>
       <c r="E5" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>2.71255060728745</v>
       </c>
       <c r="F5" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>3.58552631578947</v>
       </c>
       <c r="G5" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A5)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>4.4585020242915</v>
       </c>
     </row>
@@ -4326,23 +4581,23 @@
         <v>98</v>
       </c>
       <c r="C6" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0910931174089069</v>
       </c>
       <c r="D6" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.110070850202429</v>
       </c>
       <c r="E6" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.129048582995951</v>
       </c>
       <c r="F6" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.148026315789474</v>
       </c>
       <c r="G6" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A6)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.167004048582996</v>
       </c>
     </row>
@@ -4354,23 +4609,23 @@
         <v>69</v>
       </c>
       <c r="C7" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.781882591093117</v>
       </c>
       <c r="D7" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>1.33223684210526</v>
       </c>
       <c r="E7" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>1.88259109311741</v>
       </c>
       <c r="F7" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>2.43294534412955</v>
       </c>
       <c r="G7" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A7)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>2.9832995951417</v>
       </c>
     </row>
@@ -4382,23 +4637,23 @@
         <v>71</v>
       </c>
       <c r="C8" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0265688259109312</v>
       </c>
       <c r="D8" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0265688259109312</v>
       </c>
       <c r="E8" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0265688259109312</v>
       </c>
       <c r="F8" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0265688259109312</v>
       </c>
       <c r="G8" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A8)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0265688259109312</v>
       </c>
     </row>
@@ -4410,52 +4665,52 @@
         <v>87</v>
       </c>
       <c r="C9" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
       <c r="D9" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
       <c r="E9" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
       <c r="F9" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
       <c r="G9" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A9)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C10" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
-        <v>0.0265688259109312</v>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.00885627530364372</v>
       </c>
       <c r="D10" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
-        <v>0.0265688259109312</v>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.00885627530364372</v>
       </c>
       <c r="E10" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
-        <v>0.0265688259109312</v>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.00885627530364372</v>
       </c>
       <c r="F10" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
-        <v>0.0265688259109312</v>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.00885627530364372</v>
       </c>
       <c r="G10" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A10)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
-        <v>0.0265688259109312</v>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.00885627530364372</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4466,51 +4721,51 @@
         <v>60</v>
       </c>
       <c r="C11" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.243547570850202</v>
       </c>
       <c r="D11" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.30996963562753</v>
       </c>
       <c r="E11" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.376391700404858</v>
       </c>
       <c r="F11" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.442813765182186</v>
       </c>
       <c r="G11" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A11)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.509235829959514</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C12" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0455465587044534</v>
       </c>
       <c r="D12" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0550354251012146</v>
       </c>
       <c r="E12" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0645242914979757</v>
       </c>
       <c r="F12" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0740131578947368</v>
       </c>
       <c r="G12" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A12)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.083502024291498</v>
       </c>
     </row>
@@ -4522,23 +4777,23 @@
         <v>114</v>
       </c>
       <c r="C13" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.20748987854251</v>
       </c>
       <c r="D13" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.302378542510121</v>
       </c>
       <c r="E13" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.397267206477733</v>
       </c>
       <c r="F13" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.492155870445344</v>
       </c>
       <c r="G13" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A13)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.587044534412955</v>
       </c>
     </row>
@@ -4550,23 +4805,23 @@
         <v>106</v>
       </c>
       <c r="C14" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0657894736842105</v>
       </c>
       <c r="D14" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0942560728744939</v>
       </c>
       <c r="E14" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.122722672064777</v>
       </c>
       <c r="F14" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.151189271255061</v>
       </c>
       <c r="G14" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A14)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.179655870445344</v>
       </c>
     </row>
@@ -4578,76 +4833,160 @@
         <v>110</v>
       </c>
       <c r="C15" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0657894736842105</v>
       </c>
       <c r="D15" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.0942560728744939</v>
       </c>
       <c r="E15" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.122722672064777</v>
       </c>
       <c r="F15" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.151189271255061</v>
       </c>
       <c r="G15" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$E$2:$E$60*'ТРЗ по шагам'!$H$2:$H$60)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$60=$A15)*'ТРЗ по шагам'!$F$2:$F$60*'ТРЗ по шагам'!$H$2:$H$60))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
         <v>0.179655870445344</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
-      <c r="B16" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="C16" s="17" t="n">
-        <f aca="false">SUM(C3:C15)</f>
-        <v>3.30364372469636</v>
-      </c>
-      <c r="D16" s="17" t="n">
-        <f aca="false">SUM(D3:D15)</f>
-        <v>5.13879048582996</v>
-      </c>
-      <c r="E16" s="17" t="n">
-        <f aca="false">SUM(E3:E15)</f>
-        <v>6.97393724696356</v>
-      </c>
-      <c r="F16" s="17" t="n">
-        <f aca="false">SUM(F3:F15)</f>
-        <v>8.80908400809717</v>
-      </c>
-      <c r="G16" s="17" t="n">
-        <f aca="false">SUM(G3:G15)</f>
-        <v>10.6442307692308</v>
+      <c r="A16" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.0177125506072874</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.0177125506072874</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.0177125506072874</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.0177125506072874</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.0177125506072874</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2"/>
-      <c r="B17" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="C17" s="17" t="n">
-        <f aca="false">13*1</f>
-        <v>13</v>
-      </c>
-      <c r="D17" s="17" t="n">
-        <f aca="false">13*1</f>
-        <v>13</v>
-      </c>
-      <c r="E17" s="17" t="n">
-        <f aca="false">13*1</f>
-        <v>13</v>
-      </c>
-      <c r="F17" s="17" t="n">
-        <f aca="false">13*1</f>
-        <v>13</v>
-      </c>
-      <c r="G17" s="17" t="n">
-        <f aca="false">13*1</f>
-        <v>13</v>
+      <c r="A17" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.027834008097166</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.0373228744939271</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.0468117408906883</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.0563006072874494</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.0657894736842105</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.0354251012145749</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.0354251012145749</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.0354251012145749</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.0354251012145749</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <v>0.0354251012145749</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2"/>
+      <c r="B19" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C19" s="17" t="n">
+        <f aca="false">SUM(C3:C18)</f>
+        <v>3.3669028340081</v>
+      </c>
+      <c r="D19" s="17" t="n">
+        <f aca="false">SUM(D3:D18)</f>
+        <v>5.21153846153846</v>
+      </c>
+      <c r="E19" s="17" t="n">
+        <f aca="false">SUM(E3:E18)</f>
+        <v>7.05617408906883</v>
+      </c>
+      <c r="F19" s="17" t="n">
+        <f aca="false">SUM(F3:F18)</f>
+        <v>8.90080971659919</v>
+      </c>
+      <c r="G19" s="17" t="n">
+        <f aca="false">SUM(G3:G18)</f>
+        <v>10.7454453441296</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2"/>
+      <c r="B20" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="C20" s="17" t="n">
+        <f aca="false">16*1</f>
+        <v>16</v>
+      </c>
+      <c r="D20" s="17" t="n">
+        <f aca="false">16*1</f>
+        <v>16</v>
+      </c>
+      <c r="E20" s="17" t="n">
+        <f aca="false">16*1</f>
+        <v>16</v>
+      </c>
+      <c r="F20" s="17" t="n">
+        <f aca="false">16*1</f>
+        <v>16</v>
+      </c>
+      <c r="G20" s="17" t="n">
+        <f aca="false">16*1</f>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -4674,7 +5013,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4682,42 +5021,42 @@
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add VNP authorities: confirm release scope (0.0), demo acceptance (1.1b), PreProd check (10.1b), user communication after Prod (12.4b)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A9jLsEDeJJYPHEQRo2Ao9x
</commit_message>
<xml_diff>
--- a/docs/release-trz-fte.xlsx
+++ b/docs/release-trz-fte.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="177">
   <si>
     <t xml:space="preserve">Параметр</t>
   </si>
@@ -147,6 +147,21 @@
     <t xml:space="preserve">Часов в год</t>
   </si>
   <si>
+    <t xml:space="preserve">0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Подтверждение состава релиза ВНП</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ВНП</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Владелец направления (ВНП)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.1</t>
   </si>
   <si>
@@ -159,9 +174,6 @@
     <t xml:space="preserve">Release owner / РП</t>
   </si>
   <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
     <t xml:space="preserve">0.2</t>
   </si>
   <si>
@@ -192,6 +204,12 @@
     <t xml:space="preserve">Слияние PR по задачам Fix Version</t>
   </si>
   <si>
+    <t xml:space="preserve">1.1b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Демо и приёмка задач ВНП (по ходу закрытия)</t>
+  </si>
+  <si>
     <t xml:space="preserve">1.2</t>
   </si>
   <si>
@@ -249,12 +267,6 @@
     <t xml:space="preserve">QA / регресс UAT</t>
   </si>
   <si>
-    <t xml:space="preserve">ВНП</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Владелец направления (ВНП)</t>
-  </si>
-  <si>
     <t xml:space="preserve">4.1</t>
   </si>
   <si>
@@ -384,6 +396,12 @@
     <t xml:space="preserve">Сервис ГПН-ЦР</t>
   </si>
   <si>
+    <t xml:space="preserve">10.1b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Проверка функционала на PreProd ВНП</t>
+  </si>
+  <si>
     <t xml:space="preserve">10.2</t>
   </si>
   <si>
@@ -442,6 +460,12 @@
   </si>
   <si>
     <t xml:space="preserve">Post-release check / smoke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.4b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Коммуникация ВНП с пользователями после релиза</t>
   </si>
   <si>
     <t xml:space="preserve">12.5</t>
@@ -1182,7 +1206,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K64"/>
+  <dimension ref="A1:K68"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -1244,10 +1268,10 @@
         <v>39</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>40</v>
@@ -1258,18 +1282,18 @@
       </c>
       <c r="I2" s="7" t="n">
         <f aca="false">(E2+F2*N_SVC)*H2</f>
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="J2" s="7" t="n">
         <f aca="false">(E2*HF_F+F2)*H2</f>
-        <v>3.25</v>
+        <v>2.5</v>
       </c>
       <c r="K2" s="7" t="n">
         <f aca="false">I2*REL_YEAR+J2*HF_YEAR</f>
-        <v>115</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>41</v>
       </c>
@@ -1283,10 +1307,10 @@
         <v>44</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>40</v>
@@ -1297,32 +1321,32 @@
       </c>
       <c r="I3" s="7" t="n">
         <f aca="false">(E3+F3*N_SVC)*H3</f>
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="J3" s="7" t="n">
         <f aca="false">(E3*HF_F+F3)*H3</f>
-        <v>1</v>
+        <v>3.25</v>
       </c>
       <c r="K3" s="7" t="n">
         <f aca="false">I3*REL_YEAR+J3*HF_YEAR</f>
-        <v>76</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>0.5</v>
@@ -1336,35 +1360,35 @@
       </c>
       <c r="I4" s="7" t="n">
         <f aca="false">(E4+F4*N_SVC)*H4</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J4" s="7" t="n">
         <f aca="false">(E4*HF_F+F4)*H4</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K4" s="7" t="n">
         <f aca="false">I4*REL_YEAR+J4*HF_YEAR</f>
-        <v>62</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>40</v>
@@ -1375,7 +1399,7 @@
       </c>
       <c r="I5" s="7" t="n">
         <f aca="false">(E5+F5*N_SVC)*H5</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J5" s="7" t="n">
         <f aca="false">(E5*HF_F+F5)*H5</f>
@@ -1383,15 +1407,15 @@
       </c>
       <c r="K5" s="7" t="n">
         <f aca="false">I5*REL_YEAR+J5*HF_YEAR</f>
-        <v>14</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>43</v>
@@ -1400,7 +1424,7 @@
         <v>44</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>0</v>
@@ -1414,35 +1438,35 @@
       </c>
       <c r="I6" s="7" t="n">
         <f aca="false">(E6+F6*N_SVC)*H6</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J6" s="7" t="n">
         <f aca="false">(E6*HF_F+F6)*H6</f>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="K6" s="7" t="n">
         <f aca="false">I6*REL_YEAR+J6*HF_YEAR</f>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>40</v>
@@ -1453,35 +1477,35 @@
       </c>
       <c r="I7" s="7" t="n">
         <f aca="false">(E7+F7*N_SVC)*H7</f>
-        <v>9</v>
+        <v>0.5</v>
       </c>
       <c r="J7" s="7" t="n">
         <f aca="false">(E7*HF_F+F7)*H7</f>
-        <v>2.5</v>
+        <v>0.25</v>
       </c>
       <c r="K7" s="7" t="n">
         <f aca="false">I7*REL_YEAR+J7*HF_YEAR</f>
-        <v>118</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>40</v>
@@ -1492,35 +1516,35 @@
       </c>
       <c r="I8" s="7" t="n">
         <f aca="false">(E8+F8*N_SVC)*H8</f>
-        <v>40</v>
+        <v>9</v>
       </c>
       <c r="J8" s="7" t="n">
         <f aca="false">(E8*HF_F+F8)*H8</f>
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="K8" s="7" t="n">
         <f aca="false">I8*REL_YEAR+J8*HF_YEAR</f>
-        <v>496</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.1</v>
+        <v>4</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>40</v>
@@ -1531,35 +1555,35 @@
       </c>
       <c r="I9" s="7" t="n">
         <f aca="false">(E9+F9*N_SVC)*H9</f>
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="J9" s="7" t="n">
         <f aca="false">(E9*HF_F+F9)*H9</f>
-        <v>1.1</v>
+        <v>4</v>
       </c>
       <c r="K9" s="7" t="n">
         <f aca="false">I9*REL_YEAR+J9*HF_YEAR</f>
-        <v>40.4</v>
+        <v>496</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>40</v>
@@ -1570,35 +1594,35 @@
       </c>
       <c r="I10" s="7" t="n">
         <f aca="false">(E10+F10*N_SVC)*H10</f>
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="J10" s="7" t="n">
         <f aca="false">(E10*HF_F+F10)*H10</f>
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="K10" s="7" t="n">
         <f aca="false">I10*REL_YEAR+J10*HF_YEAR</f>
-        <v>118</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>2</v>
+        <v>0.1</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>40</v>
@@ -1609,29 +1633,29 @@
       </c>
       <c r="I11" s="7" t="n">
         <f aca="false">(E11+F11*N_SVC)*H11</f>
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="J11" s="7" t="n">
         <f aca="false">(E11*HF_F+F11)*H11</f>
-        <v>2</v>
+        <v>1.1</v>
       </c>
       <c r="K11" s="7" t="n">
         <f aca="false">I11*REL_YEAR+J11*HF_YEAR</f>
-        <v>248</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>40.4</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>4</v>
@@ -1661,22 +1685,22 @@
     </row>
     <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>40</v>
@@ -1687,29 +1711,29 @@
       </c>
       <c r="I13" s="7" t="n">
         <f aca="false">(E13+F13*N_SVC)*H13</f>
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="J13" s="7" t="n">
         <f aca="false">(E13*HF_F+F13)*H13</f>
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K13" s="7" t="n">
         <f aca="false">I13*REL_YEAR+J13*HF_YEAR</f>
-        <v>744</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>4</v>
@@ -1745,97 +1769,97 @@
         <v>62</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="H15" s="6" t="n">
         <f aca="false">IF(G15="psi",P_PSI,IF(G15="ptz",P_PTZ,1))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I15" s="7" t="n">
         <f aca="false">(E15+F15*N_SVC)*H15</f>
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="J15" s="7" t="n">
         <f aca="false">(E15*HF_F+F15)*H15</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K15" s="7" t="n">
         <f aca="false">I15*REL_YEAR+J15*HF_YEAR</f>
-        <v>56</v>
+        <v>744</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>44</v>
+        <v>66</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="H16" s="6" t="n">
         <f aca="false">IF(G16="psi",P_PSI,IF(G16="ptz",P_PTZ,1))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I16" s="7" t="n">
         <f aca="false">(E16+F16*N_SVC)*H16</f>
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J16" s="7" t="n">
         <f aca="false">(E16*HF_F+F16)*H16</f>
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="K16" s="7" t="n">
         <f aca="false">I16*REL_YEAR+J16*HF_YEAR</f>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="H17" s="6" t="n">
         <f aca="false">IF(G17="psi",P_PSI,IF(G17="ptz",P_PTZ,1))</f>
@@ -1843,38 +1867,38 @@
       </c>
       <c r="I17" s="7" t="n">
         <f aca="false">(E17+F17*N_SVC)*H17</f>
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="J17" s="7" t="n">
         <f aca="false">(E17*HF_F+F17)*H17</f>
-        <v>0.75</v>
+        <v>2</v>
       </c>
       <c r="K17" s="7" t="n">
         <f aca="false">I17*REL_YEAR+J17*HF_YEAR</f>
-        <v>21</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="H18" s="6" t="n">
         <f aca="false">IF(G18="psi",P_PSI,IF(G18="ptz",P_PTZ,1))</f>
@@ -1882,38 +1906,38 @@
       </c>
       <c r="I18" s="7" t="n">
         <f aca="false">(E18+F18*N_SVC)*H18</f>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J18" s="7" t="n">
         <f aca="false">(E18*HF_F+F18)*H18</f>
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="K18" s="7" t="n">
         <f aca="false">I18*REL_YEAR+J18*HF_YEAR</f>
-        <v>84</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="E19" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="H19" s="6" t="n">
         <f aca="false">IF(G19="psi",P_PSI,IF(G19="ptz",P_PTZ,1))</f>
@@ -1921,15 +1945,15 @@
       </c>
       <c r="I19" s="7" t="n">
         <f aca="false">(E19+F19*N_SVC)*H19</f>
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="J19" s="7" t="n">
         <f aca="false">(E19*HF_F+F19)*H19</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="K19" s="7" t="n">
         <f aca="false">I19*REL_YEAR+J19*HF_YEAR</f>
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1940,77 +1964,77 @@
         <v>73</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D20" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="E20" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F20" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>40</v>
       </c>
       <c r="H20" s="6" t="n">
         <f aca="false">IF(G20="psi",P_PSI,IF(G20="ptz",P_PTZ,1))</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I20" s="7" t="n">
         <f aca="false">(E20+F20*N_SVC)*H20</f>
-        <v>128</v>
+        <v>6</v>
       </c>
       <c r="J20" s="7" t="n">
         <f aca="false">(E20*HF_F+F20)*H20</f>
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="K20" s="7" t="n">
         <f aca="false">I20*REL_YEAR+J20*HF_YEAR</f>
-        <v>1600</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>69</v>
+        <v>39</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>4</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="H21" s="6" t="n">
         <f aca="false">IF(G21="psi",P_PSI,IF(G21="ptz",P_PTZ,1))</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I21" s="7" t="n">
         <f aca="false">(E21+F21*N_SVC)*H21</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="J21" s="7" t="n">
         <f aca="false">(E21*HF_F+F21)*H21</f>
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="K21" s="7" t="n">
         <f aca="false">I21*REL_YEAR+J21*HF_YEAR</f>
-        <v>118</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
         <v>76</v>
       </c>
@@ -2018,16 +2042,16 @@
         <v>77</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>45</v>
+        <v>74</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>40</v>
@@ -2038,15 +2062,15 @@
       </c>
       <c r="I22" s="7" t="n">
         <f aca="false">(E22+F22*N_SVC)*H22</f>
-        <v>100</v>
+        <v>128</v>
       </c>
       <c r="J22" s="7" t="n">
         <f aca="false">(E22*HF_F+F22)*H22</f>
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="K22" s="7" t="n">
         <f aca="false">I22*REL_YEAR+J22*HF_YEAR</f>
-        <v>1240</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2057,16 +2081,16 @@
         <v>79</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="G23" s="3" t="s">
         <v>40</v>
@@ -2077,18 +2101,18 @@
       </c>
       <c r="I23" s="7" t="n">
         <f aca="false">(E23+F23*N_SVC)*H23</f>
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="J23" s="7" t="n">
         <f aca="false">(E23*HF_F+F23)*H23</f>
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="K23" s="7" t="n">
         <f aca="false">I23*REL_YEAR+J23*HF_YEAR</f>
-        <v>248</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
         <v>80</v>
       </c>
@@ -2096,16 +2120,16 @@
         <v>81</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>40</v>
@@ -2116,35 +2140,35 @@
       </c>
       <c r="I24" s="7" t="n">
         <f aca="false">(E24+F24*N_SVC)*H24</f>
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="J24" s="7" t="n">
         <f aca="false">(E24*HF_F+F24)*H24</f>
-        <v>1.5</v>
+        <v>10</v>
       </c>
       <c r="K24" s="7" t="n">
         <f aca="false">I24*REL_YEAR+J24*HF_YEAR</f>
-        <v>42</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>40</v>
@@ -2155,23 +2179,23 @@
       </c>
       <c r="I25" s="7" t="n">
         <f aca="false">(E25+F25*N_SVC)*H25</f>
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="J25" s="7" t="n">
         <f aca="false">(E25*HF_F+F25)*H25</f>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="K25" s="7" t="n">
         <f aca="false">I25*REL_YEAR+J25*HF_YEAR</f>
-        <v>42</v>
+        <v>248</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>43</v>
@@ -2180,7 +2204,7 @@
         <v>44</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F26" s="3" t="n">
         <v>0</v>
@@ -2194,32 +2218,32 @@
       </c>
       <c r="I26" s="7" t="n">
         <f aca="false">(E26+F26*N_SVC)*H26</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J26" s="7" t="n">
         <f aca="false">(E26*HF_F+F26)*H26</f>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="K26" s="7" t="n">
         <f aca="false">I26*REL_YEAR+J26*HF_YEAR</f>
-        <v>28</v>
+        <v>42</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>38</v>
+        <v>74</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F27" s="3" t="n">
         <v>0</v>
@@ -2233,32 +2257,32 @@
       </c>
       <c r="I27" s="7" t="n">
         <f aca="false">(E27+F27*N_SVC)*H27</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J27" s="7" t="n">
         <f aca="false">(E27*HF_F+F27)*H27</f>
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="K27" s="7" t="n">
         <f aca="false">I27*REL_YEAR+J27*HF_YEAR</f>
-        <v>14</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F28" s="3" t="n">
         <v>0</v>
@@ -2272,32 +2296,32 @@
       </c>
       <c r="I28" s="7" t="n">
         <f aca="false">(E28+F28*N_SVC)*H28</f>
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J28" s="7" t="n">
         <f aca="false">(E28*HF_F+F28)*H28</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K28" s="7" t="n">
         <f aca="false">I28*REL_YEAR+J28*HF_YEAR</f>
-        <v>84</v>
+        <v>28</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>86</v>
+        <v>43</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>87</v>
+        <v>44</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29" s="3" t="n">
         <v>0</v>
@@ -2311,15 +2335,15 @@
       </c>
       <c r="I29" s="7" t="n">
         <f aca="false">(E29+F29*N_SVC)*H29</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J29" s="7" t="n">
         <f aca="false">(E29*HF_F+F29)*H29</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="K29" s="7" t="n">
         <f aca="false">I29*REL_YEAR+J29*HF_YEAR</f>
-        <v>28</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2336,10 +2360,10 @@
         <v>44</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="G30" s="3" t="s">
         <v>40</v>
@@ -2350,35 +2374,35 @@
       </c>
       <c r="I30" s="7" t="n">
         <f aca="false">(E30+F30*N_SVC)*H30</f>
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="J30" s="7" t="n">
         <f aca="false">(E30*HF_F+F30)*H30</f>
-        <v>1.25</v>
+        <v>3</v>
       </c>
       <c r="K30" s="7" t="n">
         <f aca="false">I30*REL_YEAR+J30*HF_YEAR</f>
-        <v>59</v>
+        <v>84</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="D31" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>60</v>
-      </c>
       <c r="E31" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G31" s="3" t="s">
         <v>40</v>
@@ -2389,35 +2413,35 @@
       </c>
       <c r="I31" s="7" t="n">
         <f aca="false">(E31+F31*N_SVC)*H31</f>
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="J31" s="7" t="n">
         <f aca="false">(E31*HF_F+F31)*H31</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K31" s="7" t="n">
         <f aca="false">I31*REL_YEAR+J31*HF_YEAR</f>
-        <v>236</v>
+        <v>28</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G32" s="3" t="s">
         <v>40</v>
@@ -2428,68 +2452,68 @@
       </c>
       <c r="I32" s="7" t="n">
         <f aca="false">(E32+F32*N_SVC)*H32</f>
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="J32" s="7" t="n">
         <f aca="false">(E32*HF_F+F32)*H32</f>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="K32" s="7" t="n">
         <f aca="false">I32*REL_YEAR+J32*HF_YEAR</f>
-        <v>28</v>
+        <v>59</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>94</v>
+        <v>40</v>
       </c>
       <c r="H33" s="6" t="n">
         <f aca="false">IF(G33="psi",P_PSI,IF(G33="ptz",P_PTZ,1))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I33" s="7" t="n">
         <f aca="false">(E33+F33*N_SVC)*H33</f>
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="J33" s="7" t="n">
         <f aca="false">(E33*HF_F+F33)*H33</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K33" s="7" t="n">
         <f aca="false">I33*REL_YEAR+J33*HF_YEAR</f>
-        <v>28</v>
+        <v>236</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E34" s="3" t="n">
         <v>2</v>
@@ -2498,101 +2522,101 @@
         <v>0</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>94</v>
+        <v>40</v>
       </c>
       <c r="H34" s="6" t="n">
         <f aca="false">IF(G34="psi",P_PSI,IF(G34="ptz",P_PTZ,1))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I34" s="7" t="n">
         <f aca="false">(E34+F34*N_SVC)*H34</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J34" s="7" t="n">
         <f aca="false">(E34*HF_F+F34)*H34</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K34" s="7" t="n">
         <f aca="false">I34*REL_YEAR+J34*HF_YEAR</f>
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>44</v>
+        <v>66</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>40</v>
+        <v>98</v>
       </c>
       <c r="H35" s="6" t="n">
         <f aca="false">IF(G35="psi",P_PSI,IF(G35="ptz",P_PTZ,1))</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I35" s="7" t="n">
         <f aca="false">(E35+F35*N_SVC)*H35</f>
-        <v>5.5</v>
+        <v>2</v>
       </c>
       <c r="J35" s="7" t="n">
         <f aca="false">(E35*HF_F+F35)*H35</f>
-        <v>1.75</v>
+        <v>1</v>
       </c>
       <c r="K35" s="7" t="n">
         <f aca="false">I35*REL_YEAR+J35*HF_YEAR</f>
-        <v>73</v>
+        <v>28</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>97</v>
+        <v>47</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F36" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>40</v>
+        <v>98</v>
       </c>
       <c r="H36" s="6" t="n">
         <f aca="false">IF(G36="psi",P_PSI,IF(G36="ptz",P_PTZ,1))</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I36" s="7" t="n">
         <f aca="false">(E36+F36*N_SVC)*H36</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J36" s="7" t="n">
         <f aca="false">(E36*HF_F+F36)*H36</f>
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="K36" s="7" t="n">
         <f aca="false">I36*REL_YEAR+J36*HF_YEAR</f>
-        <v>56</v>
+        <v>14</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2603,10 +2627,10 @@
         <v>100</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>3</v>
@@ -2642,13 +2666,13 @@
         <v>100</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>38</v>
+        <v>101</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>39</v>
+        <v>102</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F38" s="3" t="n">
         <v>0</v>
@@ -2662,35 +2686,35 @@
       </c>
       <c r="I38" s="7" t="n">
         <f aca="false">(E38+F38*N_SVC)*H38</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J38" s="7" t="n">
         <f aca="false">(E38*HF_F+F38)*H38</f>
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="K38" s="7" t="n">
         <f aca="false">I38*REL_YEAR+J38*HF_YEAR</f>
-        <v>14</v>
+        <v>56</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>98</v>
+        <v>66</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="G39" s="3" t="s">
         <v>40</v>
@@ -2701,23 +2725,23 @@
       </c>
       <c r="I39" s="7" t="n">
         <f aca="false">(E39+F39*N_SVC)*H39</f>
-        <v>9</v>
+        <v>5.5</v>
       </c>
       <c r="J39" s="7" t="n">
         <f aca="false">(E39*HF_F+F39)*H39</f>
-        <v>2.5</v>
+        <v>1.75</v>
       </c>
       <c r="K39" s="7" t="n">
         <f aca="false">I39*REL_YEAR+J39*HF_YEAR</f>
-        <v>118</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>43</v>
@@ -2729,7 +2753,7 @@
         <v>1</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>40</v>
@@ -2740,32 +2764,32 @@
       </c>
       <c r="I40" s="7" t="n">
         <f aca="false">(E40+F40*N_SVC)*H40</f>
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="J40" s="7" t="n">
         <f aca="false">(E40*HF_F+F40)*H40</f>
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="K40" s="7" t="n">
         <f aca="false">I40*REL_YEAR+J40*HF_YEAR</f>
-        <v>45</v>
+        <v>14</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F41" s="3" t="n">
         <v>0.5</v>
@@ -2779,35 +2803,35 @@
       </c>
       <c r="I41" s="7" t="n">
         <f aca="false">(E41+F41*N_SVC)*H41</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J41" s="7" t="n">
         <f aca="false">(E41*HF_F+F41)*H41</f>
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="K41" s="7" t="n">
         <f aca="false">I41*REL_YEAR+J41*HF_YEAR</f>
-        <v>90</v>
+        <v>118</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>109</v>
+        <v>47</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>110</v>
+        <v>48</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="G42" s="3" t="s">
         <v>40</v>
@@ -2818,35 +2842,35 @@
       </c>
       <c r="I42" s="7" t="n">
         <f aca="false">(E42+F42*N_SVC)*H42</f>
-        <v>7</v>
+        <v>3.5</v>
       </c>
       <c r="J42" s="7" t="n">
         <f aca="false">(E42*HF_F+F42)*H42</f>
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="K42" s="7" t="n">
         <f aca="false">I42*REL_YEAR+J42*HF_YEAR</f>
-        <v>90</v>
+        <v>45</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>38</v>
+        <v>109</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>39</v>
+        <v>110</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G43" s="3" t="s">
         <v>40</v>
@@ -2857,15 +2881,15 @@
       </c>
       <c r="I43" s="7" t="n">
         <f aca="false">(E43+F43*N_SVC)*H43</f>
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="J43" s="7" t="n">
         <f aca="false">(E43*HF_F+F43)*H43</f>
-        <v>5</v>
+        <v>1.5</v>
       </c>
       <c r="K43" s="7" t="n">
         <f aca="false">I43*REL_YEAR+J43*HF_YEAR</f>
-        <v>236</v>
+        <v>90</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2882,10 +2906,10 @@
         <v>114</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="G44" s="3" t="s">
         <v>40</v>
@@ -2896,15 +2920,15 @@
       </c>
       <c r="I44" s="7" t="n">
         <f aca="false">(E44+F44*N_SVC)*H44</f>
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="J44" s="7" t="n">
         <f aca="false">(E44*HF_F+F44)*H44</f>
-        <v>6</v>
+        <v>1.5</v>
       </c>
       <c r="K44" s="7" t="n">
         <f aca="false">I44*REL_YEAR+J44*HF_YEAR</f>
-        <v>360</v>
+        <v>90</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2915,16 +2939,16 @@
         <v>116</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45" s="3" t="s">
         <v>40</v>
@@ -2935,35 +2959,35 @@
       </c>
       <c r="I45" s="7" t="n">
         <f aca="false">(E45+F45*N_SVC)*H45</f>
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="J45" s="7" t="n">
         <f aca="false">(E45*HF_F+F45)*H45</f>
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="K45" s="7" t="n">
         <f aca="false">I45*REL_YEAR+J45*HF_YEAR</f>
-        <v>42</v>
+        <v>236</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="D46" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="C46" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>39</v>
-      </c>
       <c r="E46" s="3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G46" s="3" t="s">
         <v>40</v>
@@ -2974,35 +2998,35 @@
       </c>
       <c r="I46" s="7" t="n">
         <f aca="false">(E46+F46*N_SVC)*H46</f>
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="J46" s="7" t="n">
         <f aca="false">(E46*HF_F+F46)*H46</f>
-        <v>0.5</v>
+        <v>6</v>
       </c>
       <c r="K46" s="7" t="n">
         <f aca="false">I46*REL_YEAR+J46*HF_YEAR</f>
-        <v>14</v>
+        <v>360</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G47" s="3" t="s">
         <v>40</v>
@@ -3013,32 +3037,32 @@
       </c>
       <c r="I47" s="7" t="n">
         <f aca="false">(E47+F47*N_SVC)*H47</f>
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="J47" s="7" t="n">
         <f aca="false">(E47*HF_F+F47)*H47</f>
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="K47" s="7" t="n">
         <f aca="false">I47*REL_YEAR+J47*HF_YEAR</f>
-        <v>14</v>
+        <v>152</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>121</v>
+        <v>43</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>122</v>
+        <v>44</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F48" s="3" t="n">
         <v>0</v>
@@ -3052,29 +3076,29 @@
       </c>
       <c r="I48" s="7" t="n">
         <f aca="false">(E48+F48*N_SVC)*H48</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J48" s="7" t="n">
         <f aca="false">(E48*HF_F+F48)*H48</f>
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="K48" s="7" t="n">
         <f aca="false">I48*REL_YEAR+J48*HF_YEAR</f>
-        <v>56</v>
+        <v>42</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>123</v>
+        <v>43</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>124</v>
+        <v>44</v>
       </c>
       <c r="E49" s="3" t="n">
         <v>1</v>
@@ -3104,10 +3128,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>38</v>
@@ -3158,7 +3182,7 @@
         <v>4</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>40</v>
@@ -3169,15 +3193,15 @@
       </c>
       <c r="I51" s="7" t="n">
         <f aca="false">(E51+F51*N_SVC)*H51</f>
-        <v>6.5</v>
+        <v>4</v>
       </c>
       <c r="J51" s="7" t="n">
         <f aca="false">(E51*HF_F+F51)*H51</f>
-        <v>2.25</v>
+        <v>2</v>
       </c>
       <c r="K51" s="7" t="n">
         <f aca="false">I51*REL_YEAR+J51*HF_YEAR</f>
-        <v>87</v>
+        <v>56</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3188,13 +3212,13 @@
         <v>126</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>38</v>
+        <v>129</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>39</v>
+        <v>130</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F52" s="3" t="n">
         <v>0</v>
@@ -3208,35 +3232,35 @@
       </c>
       <c r="I52" s="7" t="n">
         <f aca="false">(E52+F52*N_SVC)*H52</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J52" s="7" t="n">
         <f aca="false">(E52*HF_F+F52)*H52</f>
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="K52" s="7" t="n">
         <f aca="false">I52*REL_YEAR+J52*HF_YEAR</f>
-        <v>42</v>
+        <v>14</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>105</v>
+        <v>43</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>106</v>
+        <v>44</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="G53" s="3" t="s">
         <v>40</v>
@@ -3247,15 +3271,15 @@
       </c>
       <c r="I53" s="7" t="n">
         <f aca="false">(E53+F53*N_SVC)*H53</f>
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="J53" s="7" t="n">
         <f aca="false">(E53*HF_F+F53)*H53</f>
-        <v>1.25</v>
+        <v>0.5</v>
       </c>
       <c r="K53" s="7" t="n">
         <f aca="false">I53*REL_YEAR+J53*HF_YEAR</f>
-        <v>59</v>
+        <v>14</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3266,13 +3290,13 @@
         <v>132</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>109</v>
+        <v>133</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>110</v>
+        <v>134</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F54" s="3" t="n">
         <v>0.25</v>
@@ -3286,35 +3310,35 @@
       </c>
       <c r="I54" s="7" t="n">
         <f aca="false">(E54+F54*N_SVC)*H54</f>
-        <v>4.5</v>
+        <v>6.5</v>
       </c>
       <c r="J54" s="7" t="n">
         <f aca="false">(E54*HF_F+F54)*H54</f>
-        <v>1.25</v>
+        <v>2.25</v>
       </c>
       <c r="K54" s="7" t="n">
         <f aca="false">I54*REL_YEAR+J54*HF_YEAR</f>
-        <v>59</v>
+        <v>87</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>113</v>
+        <v>43</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>114</v>
+        <v>44</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="G55" s="3" t="s">
         <v>40</v>
@@ -3325,15 +3349,15 @@
       </c>
       <c r="I55" s="7" t="n">
         <f aca="false">(E55+F55*N_SVC)*H55</f>
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J55" s="7" t="n">
         <f aca="false">(E55*HF_F+F55)*H55</f>
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="K55" s="7" t="n">
         <f aca="false">I55*REL_YEAR+J55*HF_YEAR</f>
-        <v>118</v>
+        <v>42</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3344,10 +3368,10 @@
         <v>136</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>43</v>
+        <v>109</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>44</v>
+        <v>110</v>
       </c>
       <c r="E56" s="3" t="n">
         <v>2</v>
@@ -3375,24 +3399,24 @@
         <v>59</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>45</v>
+        <v>113</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>46</v>
+        <v>114</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>40</v>
@@ -3403,35 +3427,35 @@
       </c>
       <c r="I57" s="7" t="n">
         <f aca="false">(E57+F57*N_SVC)*H57</f>
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="J57" s="7" t="n">
         <f aca="false">(E57*HF_F+F57)*H57</f>
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="K57" s="7" t="n">
         <f aca="false">I57*REL_YEAR+J57*HF_YEAR</f>
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>38</v>
+        <v>117</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>39</v>
+        <v>118</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G58" s="3" t="s">
         <v>40</v>
@@ -3442,32 +3466,32 @@
       </c>
       <c r="I58" s="7" t="n">
         <f aca="false">(E58+F58*N_SVC)*H58</f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="J58" s="7" t="n">
         <f aca="false">(E58*HF_F+F58)*H58</f>
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="K58" s="7" t="n">
         <f aca="false">I58*REL_YEAR+J58*HF_YEAR</f>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>139</v>
+        <v>38</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>140</v>
+        <v>39</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F59" s="3" t="n">
         <v>0</v>
@@ -3481,29 +3505,29 @@
       </c>
       <c r="I59" s="7" t="n">
         <f aca="false">(E59+F59*N_SVC)*H59</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J59" s="7" t="n">
         <f aca="false">(E59*HF_F+F59)*H59</f>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="K59" s="7" t="n">
         <f aca="false">I59*REL_YEAR+J59*HF_YEAR</f>
-        <v>28</v>
+        <v>42</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>141</v>
+        <v>47</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>142</v>
+        <v>48</v>
       </c>
       <c r="E60" s="3" t="n">
         <v>2</v>
@@ -3531,24 +3555,24 @@
         <v>59</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G61" s="3" t="s">
         <v>40</v>
@@ -3559,7 +3583,7 @@
       </c>
       <c r="I61" s="7" t="n">
         <f aca="false">(E61+F61*N_SVC)*H61</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J61" s="7" t="n">
         <f aca="false">(E61*HF_F+F61)*H61</f>
@@ -3567,24 +3591,24 @@
       </c>
       <c r="K61" s="7" t="n">
         <f aca="false">I61*REL_YEAR+J61*HF_YEAR</f>
-        <v>14</v>
+        <v>62</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F62" s="3" t="n">
         <v>0</v>
@@ -3598,32 +3622,32 @@
       </c>
       <c r="I62" s="7" t="n">
         <f aca="false">(E62+F62*N_SVC)*H62</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J62" s="7" t="n">
         <f aca="false">(E62*HF_F+F62)*H62</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K62" s="7" t="n">
         <f aca="false">I62*REL_YEAR+J62*HF_YEAR</f>
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>59</v>
+        <v>147</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>60</v>
+        <v>148</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F63" s="3" t="n">
         <v>0</v>
@@ -3637,39 +3661,195 @@
       </c>
       <c r="I63" s="7" t="n">
         <f aca="false">(E63+F63*N_SVC)*H63</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J63" s="7" t="n">
         <f aca="false">(E63*HF_F+F63)*H63</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K63" s="7" t="n">
         <f aca="false">I63*REL_YEAR+J63*HF_YEAR</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G64" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H64" s="6" t="n">
+        <f aca="false">IF(G64="psi",P_PSI,IF(G64="ptz",P_PTZ,1))</f>
+        <v>1</v>
+      </c>
+      <c r="I64" s="7" t="n">
+        <f aca="false">(E64+F64*N_SVC)*H64</f>
+        <v>4.5</v>
+      </c>
+      <c r="J64" s="7" t="n">
+        <f aca="false">(E64*HF_F+F64)*H64</f>
+        <v>1.25</v>
+      </c>
+      <c r="K64" s="7" t="n">
+        <f aca="false">I64*REL_YEAR+J64*HF_YEAR</f>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H65" s="6" t="n">
+        <f aca="false">IF(G65="psi",P_PSI,IF(G65="ptz",P_PTZ,1))</f>
+        <v>1</v>
+      </c>
+      <c r="I65" s="7" t="n">
+        <f aca="false">(E65+F65*N_SVC)*H65</f>
+        <v>1</v>
+      </c>
+      <c r="J65" s="7" t="n">
+        <f aca="false">(E65*HF_F+F65)*H65</f>
+        <v>0.5</v>
+      </c>
+      <c r="K65" s="7" t="n">
+        <f aca="false">I65*REL_YEAR+J65*HF_YEAR</f>
         <v>14</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="2"/>
-      <c r="B64" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="C64" s="2"/>
-      <c r="D64" s="2"/>
-      <c r="E64" s="2"/>
-      <c r="F64" s="2"/>
-      <c r="G64" s="2"/>
-      <c r="H64" s="6"/>
-      <c r="I64" s="9" t="n">
-        <f aca="false">SUM(I2:I63)</f>
-        <v>644</v>
-      </c>
-      <c r="J64" s="9" t="n">
-        <f aca="false">SUM(J2:J63)</f>
-        <v>127.6</v>
-      </c>
-      <c r="K64" s="9" t="n">
-        <f aca="false">SUM(K2:K63)</f>
-        <v>8238.4</v>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H66" s="6" t="n">
+        <f aca="false">IF(G66="psi",P_PSI,IF(G66="ptz",P_PTZ,1))</f>
+        <v>1</v>
+      </c>
+      <c r="I66" s="7" t="n">
+        <f aca="false">(E66+F66*N_SVC)*H66</f>
+        <v>1</v>
+      </c>
+      <c r="J66" s="7" t="n">
+        <f aca="false">(E66*HF_F+F66)*H66</f>
+        <v>0.5</v>
+      </c>
+      <c r="K66" s="7" t="n">
+        <f aca="false">I66*REL_YEAR+J66*HF_YEAR</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H67" s="6" t="n">
+        <f aca="false">IF(G67="psi",P_PSI,IF(G67="ptz",P_PTZ,1))</f>
+        <v>1</v>
+      </c>
+      <c r="I67" s="7" t="n">
+        <f aca="false">(E67+F67*N_SVC)*H67</f>
+        <v>1</v>
+      </c>
+      <c r="J67" s="7" t="n">
+        <f aca="false">(E67*HF_F+F67)*H67</f>
+        <v>0.5</v>
+      </c>
+      <c r="K67" s="7" t="n">
+        <f aca="false">I67*REL_YEAR+J67*HF_YEAR</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="2"/>
+      <c r="B68" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="C68" s="2"/>
+      <c r="D68" s="2"/>
+      <c r="E68" s="2"/>
+      <c r="F68" s="2"/>
+      <c r="G68" s="2"/>
+      <c r="H68" s="6"/>
+      <c r="I68" s="9" t="n">
+        <f aca="false">SUM(I2:I67)</f>
+        <v>683</v>
+      </c>
+      <c r="J68" s="9" t="n">
+        <f aca="false">SUM(J2:J67)</f>
+        <v>135.1</v>
+      </c>
+      <c r="K68" s="9" t="n">
+        <f aca="false">SUM(K2:K67)</f>
+        <v>8736.4</v>
       </c>
     </row>
   </sheetData>
@@ -3717,40 +3897,40 @@
         <v>35</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C2" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A2)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A2)</f>
         <v>51.5</v>
       </c>
       <c r="D2" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A2)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A2)</f>
         <v>699.4</v>
       </c>
       <c r="E2" s="6" t="n">
@@ -3780,17 +3960,17 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C3" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A3)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A3)</f>
         <v>58.5</v>
       </c>
       <c r="D3" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A3)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A3)</f>
         <v>771</v>
       </c>
       <c r="E3" s="6" t="n">
@@ -3820,17 +4000,17 @@
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C4" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A4)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A4)</f>
         <v>234</v>
       </c>
       <c r="D4" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A4)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A4)</f>
         <v>2908</v>
       </c>
       <c r="E4" s="6" t="n">
@@ -3860,17 +4040,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C5" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A5)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A5)</f>
         <v>13</v>
       </c>
       <c r="D5" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A5)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A5)</f>
         <v>174</v>
       </c>
       <c r="E5" s="6" t="n">
@@ -3900,17 +4080,17 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C6" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A6)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A6)</f>
         <v>167</v>
       </c>
       <c r="D6" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A6)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A6)</f>
         <v>2106</v>
       </c>
       <c r="E6" s="6" t="n">
@@ -3940,29 +4120,29 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="C7" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A7)</f>
-        <v>3</v>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A7)</f>
+        <v>42</v>
       </c>
       <c r="D7" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A7)</f>
-        <v>42</v>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A7)</f>
+        <v>540</v>
       </c>
       <c r="E7" s="6" t="n">
         <f aca="false">D7/H_FTE</f>
-        <v>0.0265688259109312</v>
+        <v>0.341599190283401</v>
       </c>
       <c r="F7" s="11" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="6" t="n">
         <f aca="false">F7-E7</f>
-        <v>0.973431174089069</v>
+        <v>0.658400809716599</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="12" t="str">
@@ -3980,17 +4160,17 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C8" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A8)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A8)</f>
         <v>2</v>
       </c>
       <c r="D8" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A8)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A8)</f>
         <v>28</v>
       </c>
       <c r="E8" s="6" t="n">
@@ -4020,17 +4200,17 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C9" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A9)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A9)</f>
         <v>1</v>
       </c>
       <c r="D9" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A9)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A9)</f>
         <v>14</v>
       </c>
       <c r="E9" s="6" t="n">
@@ -4060,17 +4240,17 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C10" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A10)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A10)</f>
         <v>37</v>
       </c>
       <c r="D10" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A10)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A10)</f>
         <v>490</v>
       </c>
       <c r="E10" s="6" t="n">
@@ -4100,17 +4280,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="C11" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A11)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A11)</f>
         <v>6.5</v>
       </c>
       <c r="D11" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A11)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A11)</f>
         <v>87</v>
       </c>
       <c r="E11" s="6" t="n">
@@ -4140,17 +4320,17 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C12" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A12)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A12)</f>
         <v>37</v>
       </c>
       <c r="D12" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A12)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A12)</f>
         <v>478</v>
       </c>
       <c r="E12" s="6" t="n">
@@ -4180,17 +4360,17 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C13" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A13)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A13)</f>
         <v>11.5</v>
       </c>
       <c r="D13" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A13)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A13)</f>
         <v>149</v>
       </c>
       <c r="E13" s="6" t="n">
@@ -4220,17 +4400,17 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C14" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A14)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A14)</f>
         <v>11.5</v>
       </c>
       <c r="D14" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A14)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A14)</f>
         <v>149</v>
       </c>
       <c r="E14" s="6" t="n">
@@ -4260,17 +4440,17 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="C15" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A15)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A15)</f>
         <v>2</v>
       </c>
       <c r="D15" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A15)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A15)</f>
         <v>28</v>
       </c>
       <c r="E15" s="6" t="n">
@@ -4300,17 +4480,17 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="C16" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A16)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A16)</f>
         <v>4.5</v>
       </c>
       <c r="D16" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A16)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A16)</f>
         <v>59</v>
       </c>
       <c r="E16" s="6" t="n">
@@ -4340,17 +4520,17 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C17" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$63,'ТРЗ по шагам'!$C$2:$C$63,A17)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$I$2:$I$67,'ТРЗ по шагам'!$C$2:$C$67,A17)</f>
         <v>4</v>
       </c>
       <c r="D17" s="10" t="n">
-        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$63,'ТРЗ по шагам'!$C$2:$C$63,A17)</f>
+        <f aca="false">SUMIFS('ТРЗ по шагам'!$K$2:$K$67,'ТРЗ по шагам'!$C$2:$C$67,A17)</f>
         <v>56</v>
       </c>
       <c r="E17" s="6" t="n">
@@ -4381,19 +4561,19 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2"/>
       <c r="B18" s="8" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="C18" s="13" t="n">
         <f aca="false">SUM(C2:C17)</f>
-        <v>644</v>
+        <v>683</v>
       </c>
       <c r="D18" s="13" t="n">
         <f aca="false">SUM(D2:D17)</f>
-        <v>8238.4</v>
+        <v>8736.4</v>
       </c>
       <c r="E18" s="14" t="n">
         <f aca="false">SUM(E2:E17)</f>
-        <v>5.21153846153846</v>
+        <v>5.52656882591093</v>
       </c>
       <c r="F18" s="14" t="n">
         <f aca="false">SUM(F2:F17)</f>
@@ -4401,7 +4581,7 @@
       </c>
       <c r="G18" s="14" t="n">
         <f aca="false">SUM(G2:G17)</f>
-        <v>10.7884615384615</v>
+        <v>10.4734311740891</v>
       </c>
       <c r="H18" s="2"/>
       <c r="I18" s="15" t="n">
@@ -4419,7 +4599,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -4454,24 +4634,24 @@
         <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="C2" s="16" t="n">
         <v>5</v>
@@ -4491,482 +4671,482 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C3" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.391194331983806</v>
       </c>
       <c r="D3" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.442434210526316</v>
       </c>
       <c r="E3" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.493674089068826</v>
       </c>
       <c r="F3" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.544913967611336</v>
       </c>
       <c r="G3" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A3)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A3)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.596153846153846</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C4" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.373861336032389</v>
       </c>
       <c r="D4" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.487727732793522</v>
       </c>
       <c r="E4" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.601594129554656</v>
       </c>
       <c r="F4" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.715460526315789</v>
       </c>
       <c r="G4" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A4)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A4)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.829326923076923</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C5" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.966599190283401</v>
       </c>
       <c r="D5" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>1.83957489878542</v>
       </c>
       <c r="E5" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>2.71255060728745</v>
       </c>
       <c r="F5" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>3.58552631578947</v>
       </c>
       <c r="G5" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A5)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A5)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>4.4585020242915</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C6" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0910931174089069</v>
       </c>
       <c r="D6" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.110070850202429</v>
       </c>
       <c r="E6" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.129048582995951</v>
       </c>
       <c r="F6" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.148026315789474</v>
       </c>
       <c r="G6" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A6)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A6)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.167004048582996</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C7" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.781882591093117</v>
       </c>
       <c r="D7" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>1.33223684210526</v>
       </c>
       <c r="E7" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>1.88259109311741</v>
       </c>
       <c r="F7" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>2.43294534412955</v>
       </c>
       <c r="G7" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A7)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A7)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>2.9832995951417</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="C8" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
-        <v>0.0265688259109312</v>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
+        <v>0.227732793522267</v>
       </c>
       <c r="D8" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
-        <v>0.0265688259109312</v>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
+        <v>0.341599190283401</v>
       </c>
       <c r="E8" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
-        <v>0.0265688259109312</v>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
+        <v>0.455465587044534</v>
       </c>
       <c r="F8" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
-        <v>0.0265688259109312</v>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
+        <v>0.569331983805668</v>
       </c>
       <c r="G8" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A8)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
-        <v>0.0265688259109312</v>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A8)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
+        <v>0.683198380566802</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C9" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
       <c r="D9" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
       <c r="E9" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
       <c r="F9" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
       <c r="G9" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A9)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A9)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C10" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.00885627530364372</v>
       </c>
       <c r="D10" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.00885627530364372</v>
       </c>
       <c r="E10" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.00885627530364372</v>
       </c>
       <c r="F10" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.00885627530364372</v>
       </c>
       <c r="G10" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A10)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A10)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.00885627530364372</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C11" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.243547570850202</v>
       </c>
       <c r="D11" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.30996963562753</v>
       </c>
       <c r="E11" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.376391700404858</v>
       </c>
       <c r="F11" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.442813765182186</v>
       </c>
       <c r="G11" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A11)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A11)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.509235829959514</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="C12" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0455465587044534</v>
       </c>
       <c r="D12" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0550354251012146</v>
       </c>
       <c r="E12" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0645242914979757</v>
       </c>
       <c r="F12" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0740131578947368</v>
       </c>
       <c r="G12" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A12)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A12)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.083502024291498</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C13" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.20748987854251</v>
       </c>
       <c r="D13" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.302378542510121</v>
       </c>
       <c r="E13" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.397267206477733</v>
       </c>
       <c r="F13" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.492155870445344</v>
       </c>
       <c r="G13" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A13)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A13)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.587044534412955</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C14" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0657894736842105</v>
       </c>
       <c r="D14" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0942560728744939</v>
       </c>
       <c r="E14" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.122722672064777</v>
       </c>
       <c r="F14" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.151189271255061</v>
       </c>
       <c r="G14" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A14)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A14)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.179655870445344</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C15" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0657894736842105</v>
       </c>
       <c r="D15" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0942560728744939</v>
       </c>
       <c r="E15" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.122722672064777</v>
       </c>
       <c r="F15" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.151189271255061</v>
       </c>
       <c r="G15" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A15)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A15)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.179655870445344</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="C16" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
       <c r="D16" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
       <c r="E16" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
       <c r="F16" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
       <c r="G16" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A16)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A16)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0177125506072874</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="C17" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.027834008097166</v>
       </c>
       <c r="D17" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0373228744939271</v>
       </c>
       <c r="E17" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0468117408906883</v>
       </c>
       <c r="F17" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0563006072874494</v>
       </c>
       <c r="G17" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A17)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A17)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0657894736842105</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C18" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*C$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0354251012145749</v>
       </c>
       <c r="D18" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*D$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0354251012145749</v>
       </c>
       <c r="E18" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*E$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0354251012145749</v>
       </c>
       <c r="F18" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*F$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0354251012145749</v>
       </c>
       <c r="G18" s="6" t="n">
-        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$E$2:$E$63*'ТРЗ по шагам'!$H$2:$H$63)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$63=$A18)*'ТРЗ по шагам'!$F$2:$F$63*'ТРЗ по шагам'!$H$2:$H$63))*HF_YEAR)/H_FTE</f>
+        <f aca="false">((SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67)*G$2)*REL_YEAR+(SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$E$2:$E$67*'ТРЗ по шагам'!$H$2:$H$67)*HF_F+SUMPRODUCT(('ТРЗ по шагам'!$C$2:$C$67=$A18)*'ТРЗ по шагам'!$F$2:$F$67*'ТРЗ по шагам'!$H$2:$H$67))*HF_YEAR)/H_FTE</f>
         <v>0.0354251012145749</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2"/>
       <c r="B19" s="8" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="C19" s="17" t="n">
         <f aca="false">SUM(C3:C18)</f>
-        <v>3.3669028340081</v>
+        <v>3.56806680161943</v>
       </c>
       <c r="D19" s="17" t="n">
         <f aca="false">SUM(D3:D18)</f>
-        <v>5.21153846153846</v>
+        <v>5.52656882591093</v>
       </c>
       <c r="E19" s="17" t="n">
         <f aca="false">SUM(E3:E18)</f>
-        <v>7.05617408906883</v>
+        <v>7.48507085020243</v>
       </c>
       <c r="F19" s="17" t="n">
         <f aca="false">SUM(F3:F18)</f>
-        <v>8.90080971659919</v>
+        <v>9.44357287449393</v>
       </c>
       <c r="G19" s="17" t="n">
         <f aca="false">SUM(G3:G18)</f>
-        <v>10.7454453441296</v>
+        <v>11.4020748987854</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2"/>
       <c r="B20" s="8" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="C20" s="17" t="n">
         <f aca="false">16*1</f>
@@ -5013,7 +5193,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5021,42 +5201,42 @@
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>